<commit_message>
excel: q4 calculations (Manuel)
</commit_message>
<xml_diff>
--- a/Network_Data/46705_excel_task1.xlsx
+++ b/Network_Data/46705_excel_task1.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://dtudk-my.sharepoint.com/personal/s253262_dtu_dk/Documents/Documents/00_TRAVAIL/DTU/COURSES/46705_Power_Grid_Analysis/PGA_assignment_1/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/d6292b491a055b72/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3" documentId="108_{8B7BFC02-C874-4F3D-BCCF-A3DD201EEACC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{402C0AF1-22E3-4DDF-96A8-296115066E19}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{6677D636-8AAD-41DF-AB16-24D0B2B2828A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" xr2:uid="{C24A2377-180A-4C78-8908-403D56B61C41}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{C24A2377-180A-4C78-8908-403D56B61C41}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="46">
   <si>
     <t>S_base (MVA)</t>
   </si>
@@ -68,9 +68,6 @@
     <t>lenght(km)</t>
   </si>
   <si>
-    <t>ser_impedance(omh)</t>
-  </si>
-  <si>
     <t>ser_impedance(p.u.)</t>
   </si>
   <si>
@@ -126,13 +123,64 @@
   </si>
   <si>
     <t>S_low(pu)</t>
+  </si>
+  <si>
+    <t>Cable selected</t>
+  </si>
+  <si>
+    <t>C (microF/km)</t>
+  </si>
+  <si>
+    <t>Ind (mH/km)</t>
+  </si>
+  <si>
+    <t>4-&gt;6</t>
+  </si>
+  <si>
+    <t>4-&gt;5</t>
+  </si>
+  <si>
+    <t>Line</t>
+  </si>
+  <si>
+    <t>Lenght(km)</t>
+  </si>
+  <si>
+    <t>R(ohm)</t>
+  </si>
+  <si>
+    <t>C(microF)</t>
+  </si>
+  <si>
+    <t>Ind(mH)</t>
+  </si>
+  <si>
+    <t>X (omh)</t>
+  </si>
+  <si>
+    <t>Y_shant(S)</t>
+  </si>
+  <si>
+    <t>R(ohm/km)</t>
+  </si>
+  <si>
+    <t>ser_impedance(ohm)</t>
+  </si>
+  <si>
+    <t>P.u. Values</t>
+  </si>
+  <si>
+    <t>1x800RM</t>
+  </si>
+  <si>
+    <t>Copper</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -161,8 +209,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -178,6 +229,99 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>12451</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>149411</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>22</xdr:col>
+      <xdr:colOff>347104</xdr:colOff>
+      <xdr:row>68</xdr:row>
+      <xdr:rowOff>11280</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E08007F5-4EA7-3FE4-4216-A5B0508D7869}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="9126569" y="5378823"/>
+          <a:ext cx="9162398" cy="7332457"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>24</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>29</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>39</xdr:col>
+      <xdr:colOff>43610</xdr:colOff>
+      <xdr:row>85</xdr:row>
+      <xdr:rowOff>148915</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="Picture 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C21BB4D0-62EA-93D9-C8F8-84E7D3581EB9}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="19120556" y="5319889"/>
+          <a:ext cx="9145276" cy="10421804"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -497,24 +641,24 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2470A2DB-7C0C-4DC7-9EB6-537CECC5E3A8}">
-  <dimension ref="A1:S22"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:S31"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="14.140625" customWidth="1"/>
-    <col min="2" max="2" width="11.28515625" customWidth="1"/>
-    <col min="3" max="3" width="17.140625" customWidth="1"/>
-    <col min="4" max="4" width="15.85546875" customWidth="1"/>
-    <col min="5" max="5" width="16.7109375" customWidth="1"/>
+    <col min="1" max="1" width="14.1796875" customWidth="1"/>
+    <col min="2" max="2" width="12.7265625" customWidth="1"/>
+    <col min="3" max="3" width="17.1796875" customWidth="1"/>
+    <col min="4" max="4" width="15.81640625" customWidth="1"/>
+    <col min="5" max="5" width="16.7265625" customWidth="1"/>
     <col min="8" max="8" width="17" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="10.7109375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="19.140625" customWidth="1"/>
-    <col min="12" max="12" width="30.85546875" customWidth="1"/>
-    <col min="14" max="14" width="17.28515625" customWidth="1"/>
-    <col min="15" max="15" width="9.7109375" customWidth="1"/>
-    <col min="16" max="16" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.7265625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="19.1796875" customWidth="1"/>
+    <col min="12" max="12" width="8.81640625" customWidth="1"/>
+    <col min="14" max="14" width="17.26953125" customWidth="1"/>
+    <col min="15" max="15" width="9.7265625" customWidth="1"/>
+    <col min="16" max="16" width="10.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:17">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -535,7 +679,7 @@
         <v>0,08+0,5i</v>
       </c>
     </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:17">
       <c r="A2">
         <v>100</v>
       </c>
@@ -555,7 +699,7 @@
         <v>3.3</v>
       </c>
     </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:17">
       <c r="B3" t="s">
         <v>6</v>
       </c>
@@ -572,7 +716,7 @@
         <v>529</v>
       </c>
     </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:17">
       <c r="H5" t="s">
         <v>7</v>
       </c>
@@ -583,28 +727,28 @@
         <v>9</v>
       </c>
       <c r="K5" t="s">
+        <v>42</v>
+      </c>
+      <c r="L5" t="s">
         <v>10</v>
       </c>
-      <c r="L5" t="s">
+      <c r="M5" t="s">
         <v>11</v>
       </c>
-      <c r="M5" t="s">
+      <c r="N5" t="s">
         <v>12</v>
       </c>
-      <c r="N5" t="s">
+      <c r="O5" t="s">
         <v>13</v>
       </c>
-      <c r="O5" t="s">
+      <c r="P5" t="s">
         <v>14</v>
       </c>
-      <c r="P5" t="s">
+      <c r="Q5" t="s">
         <v>15</v>
       </c>
-      <c r="Q5" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="6" spans="1:17">
       <c r="H6">
         <v>1</v>
       </c>
@@ -616,7 +760,7 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:17">
       <c r="H7">
         <v>2</v>
       </c>
@@ -655,7 +799,19 @@
         <v>5.2370999999999994E-2</v>
       </c>
     </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:17">
+      <c r="B8" t="s">
+        <v>29</v>
+      </c>
+      <c r="C8" t="s">
+        <v>41</v>
+      </c>
+      <c r="D8" t="s">
+        <v>30</v>
+      </c>
+      <c r="E8" t="s">
+        <v>31</v>
+      </c>
       <c r="H8">
         <v>3</v>
       </c>
@@ -695,7 +851,22 @@
         <v>0.13267319999999999</v>
       </c>
     </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:17">
+      <c r="A9" t="s">
+        <v>45</v>
+      </c>
+      <c r="B9" t="s">
+        <v>44</v>
+      </c>
+      <c r="C9">
+        <v>2.2100000000000002E-2</v>
+      </c>
+      <c r="D9">
+        <v>0.16400000000000001</v>
+      </c>
+      <c r="E9">
+        <v>0.58099999999999996</v>
+      </c>
       <c r="H9">
         <v>4</v>
       </c>
@@ -734,7 +905,7 @@
         <v>0.13965599999999997</v>
       </c>
     </row>
-    <row r="10" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:17">
       <c r="H10">
         <v>4</v>
       </c>
@@ -773,7 +944,7 @@
         <v>5.2370999999999994E-2</v>
       </c>
     </row>
-    <row r="11" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:17">
       <c r="H11">
         <v>5</v>
       </c>
@@ -812,7 +983,7 @@
         <v>0.17457</v>
       </c>
     </row>
-    <row r="12" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:17">
       <c r="H12">
         <v>6</v>
       </c>
@@ -824,54 +995,54 @@
         <v>0.05</v>
       </c>
     </row>
-    <row r="16" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:17">
       <c r="I16" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="J16">
         <f>0.2+8*0.01</f>
         <v>0.28000000000000003</v>
       </c>
     </row>
-    <row r="17" spans="8:19" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:19">
       <c r="H17" t="s">
+        <v>17</v>
+      </c>
+      <c r="I17" t="s">
         <v>18</v>
       </c>
-      <c r="I17" t="s">
+      <c r="J17" t="s">
         <v>19</v>
       </c>
-      <c r="J17" t="s">
+      <c r="K17" t="s">
         <v>20</v>
       </c>
-      <c r="K17" t="s">
+      <c r="L17" t="s">
         <v>21</v>
       </c>
-      <c r="L17" t="s">
+      <c r="M17" t="s">
         <v>22</v>
       </c>
-      <c r="M17" t="s">
+      <c r="N17" t="s">
         <v>23</v>
       </c>
-      <c r="N17" t="s">
+      <c r="O17" t="s">
         <v>24</v>
       </c>
-      <c r="O17" t="s">
+      <c r="P17" t="s">
         <v>25</v>
       </c>
-      <c r="P17" t="s">
+      <c r="Q17" t="s">
         <v>26</v>
       </c>
-      <c r="Q17" t="s">
+      <c r="R17" t="s">
         <v>27</v>
       </c>
-      <c r="R17" t="s">
+      <c r="S17" t="s">
         <v>28</v>
       </c>
-      <c r="S17" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="18" spans="8:19" x14ac:dyDescent="0.25">
+    </row>
+    <row r="18" spans="1:19">
       <c r="H18">
         <v>2</v>
       </c>
@@ -920,7 +1091,7 @@
         <v>0.1632666530556684</v>
       </c>
     </row>
-    <row r="19" spans="8:19" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:19">
       <c r="H19">
         <v>3</v>
       </c>
@@ -969,7 +1140,7 @@
         <v>0.1632666530556684</v>
       </c>
     </row>
-    <row r="20" spans="8:19" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:19">
       <c r="H20">
         <v>4</v>
       </c>
@@ -1018,7 +1189,7 @@
         <v>0.1632666530556684</v>
       </c>
     </row>
-    <row r="21" spans="8:19" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:19">
       <c r="H21">
         <v>5</v>
       </c>
@@ -1067,7 +1238,7 @@
         <v>0.1632666530556684</v>
       </c>
     </row>
-    <row r="22" spans="8:19" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:19">
       <c r="H22">
         <v>6</v>
       </c>
@@ -1116,8 +1287,139 @@
         <v>0.1632666530556684</v>
       </c>
     </row>
+    <row r="26" spans="1:19">
+      <c r="A26" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B26" t="s">
+        <v>35</v>
+      </c>
+      <c r="C26" t="s">
+        <v>36</v>
+      </c>
+      <c r="D26" t="s">
+        <v>37</v>
+      </c>
+      <c r="E26" t="s">
+        <v>38</v>
+      </c>
+      <c r="F26" t="s">
+        <v>39</v>
+      </c>
+      <c r="G26" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="27" spans="1:19">
+      <c r="A27" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B27">
+        <v>40</v>
+      </c>
+      <c r="C27">
+        <f>$B$27*C9</f>
+        <v>0.88400000000000012</v>
+      </c>
+      <c r="D27">
+        <f>$B$27*D9</f>
+        <v>6.5600000000000005</v>
+      </c>
+      <c r="E27">
+        <f>$B$27*E9</f>
+        <v>23.24</v>
+      </c>
+      <c r="F27">
+        <f>2*PI()*50*E27*0.001</f>
+        <v>7.3010613269426798</v>
+      </c>
+      <c r="G27">
+        <f>2*PI()*50*D27*0.000001</f>
+        <v>2.0608847807549045E-3</v>
+      </c>
+    </row>
+    <row r="28" spans="1:19">
+      <c r="A28" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B28">
+        <v>15</v>
+      </c>
+      <c r="C28">
+        <f>$B$28*C9</f>
+        <v>0.33150000000000002</v>
+      </c>
+      <c r="D28">
+        <f>$B$28*D9</f>
+        <v>2.46</v>
+      </c>
+      <c r="E28">
+        <f>$B$28*E9</f>
+        <v>8.7149999999999999</v>
+      </c>
+      <c r="F28">
+        <f>2*PI()*50*E28*0.001</f>
+        <v>2.7378979976035049</v>
+      </c>
+      <c r="G28">
+        <f>2*PI()*50*D28*0.000001</f>
+        <v>7.7283179278308904E-4</v>
+      </c>
+    </row>
+    <row r="29" spans="1:19">
+      <c r="A29" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="H29" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="30" spans="1:19">
+      <c r="A30" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C30">
+        <f>C27/$E$2</f>
+        <v>3.8434782608695655E-3</v>
+      </c>
+      <c r="F30">
+        <f>F27/$E$3</f>
+        <v>1.3801628217282948E-2</v>
+      </c>
+      <c r="G30">
+        <f>G27*$E$3</f>
+        <v>1.0902080490193444</v>
+      </c>
+      <c r="H30">
+        <f>G30*2</f>
+        <v>2.1804160980386889</v>
+      </c>
+    </row>
+    <row r="31" spans="1:19">
+      <c r="A31" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="C31">
+        <f>C28/$E$2</f>
+        <v>1.441304347826087E-3</v>
+      </c>
+      <c r="F31">
+        <f>F28/$E$3</f>
+        <v>5.1756105814811061E-3</v>
+      </c>
+      <c r="G31">
+        <f>G28*$E$3</f>
+        <v>0.40882801838225408</v>
+      </c>
+      <c r="H31">
+        <f>G31*2</f>
+        <v>0.81765603676450815</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -1285,8 +1587,15 @@
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DDF9B8E9-B4B8-43C5-9789-E65419656A05}">
   <ds:schemaRefs>
+    <ds:schemaRef ds:uri="2b71e9e4-c68b-4146-8f09-a0e89ca1298a"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>